<commit_message>
Add KaTeX support for chemical formulas and math notation
- Install KaTeX library for math rendering
- Create katexRenderer utility with KatexText component
- Update CalculatorRow to render labels and units with KaTeX
- Update CalculatorGrid to render section/subsection headers with KaTeX
- Update CalculatorSelector to render calculator names/descriptions with KaTeX
- Update App.tsx to render title with KaTeX
- Update template documentation with KaTeX formatting examples

Chemical formulas updated in CSVs:
- KaKb_Determination: $[H^+]$, $[OH^-]$, $K_{eq}$, $HC_2H_3O_2$, etc.
- Separation of a Mixture: $NaI$, $NH_4Cl$, $NaCl$
- Titration: $H_2X$, $K_{a1}$, $K_{a2}$, $NaOH$
- Colligative Properties: $K_f$
- Quant Prep Gas: $H_2$, $Mg$

Usage: Wrap text in $ signs for math mode: $H_2O$ displays as H₂O
</commit_message>
<xml_diff>
--- a/Excel Logic/Colligative Properties Key CSV_HeaderBased.xlsx
+++ b/Excel Logic/Colligative Properties Key CSV_HeaderBased.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkawagoe/Scripts/Lab Check/KaKb Lab/Excel Logic/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDE4E22B-DD04-8D44-B21D-18AF690AAEB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF6E9A09-E426-F546-B083-04AF1F7A9513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="800" windowWidth="36000" windowHeight="22580" xr2:uid="{0CE90DC6-9C91-144C-A695-99A293ED696C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="58">
   <si>
     <t>Mass of test tube+beaker</t>
   </si>
@@ -259,228 +259,6 @@
   </si>
   <si>
     <t>%</t>
-  </si>
-  <si>
-    <t>F4</t>
-  </si>
-  <si>
-    <t>F5</t>
-  </si>
-  <si>
-    <t>F6</t>
-  </si>
-  <si>
-    <t>F7</t>
-  </si>
-  <si>
-    <t>F8</t>
-  </si>
-  <si>
-    <t>F9</t>
-  </si>
-  <si>
-    <t>F11</t>
-  </si>
-  <si>
-    <t>F12</t>
-  </si>
-  <si>
-    <t>F13</t>
-  </si>
-  <si>
-    <t>F14</t>
-  </si>
-  <si>
-    <t>F15</t>
-  </si>
-  <si>
-    <t>F16</t>
-  </si>
-  <si>
-    <t>F18</t>
-  </si>
-  <si>
-    <t>F19</t>
-  </si>
-  <si>
-    <t>F20</t>
-  </si>
-  <si>
-    <t>F21</t>
-  </si>
-  <si>
-    <t>F22</t>
-  </si>
-  <si>
-    <t>F23</t>
-  </si>
-  <si>
-    <t>F24</t>
-  </si>
-  <si>
-    <t>F25</t>
-  </si>
-  <si>
-    <t>F27</t>
-  </si>
-  <si>
-    <t>F28</t>
-  </si>
-  <si>
-    <t>F29</t>
-  </si>
-  <si>
-    <t>F30</t>
-  </si>
-  <si>
-    <t>F31</t>
-  </si>
-  <si>
-    <t>F32</t>
-  </si>
-  <si>
-    <t>F33</t>
-  </si>
-  <si>
-    <t>F36</t>
-  </si>
-  <si>
-    <t>F37</t>
-  </si>
-  <si>
-    <t>F38</t>
-  </si>
-  <si>
-    <t>F39</t>
-  </si>
-  <si>
-    <t>F40</t>
-  </si>
-  <si>
-    <t>F41</t>
-  </si>
-  <si>
-    <t>F42</t>
-  </si>
-  <si>
-    <t>F43</t>
-  </si>
-  <si>
-    <t>F45</t>
-  </si>
-  <si>
-    <t>F46</t>
-  </si>
-  <si>
-    <t>E4</t>
-  </si>
-  <si>
-    <t>E5</t>
-  </si>
-  <si>
-    <t>E6</t>
-  </si>
-  <si>
-    <t>E7</t>
-  </si>
-  <si>
-    <t>E8</t>
-  </si>
-  <si>
-    <t>E9</t>
-  </si>
-  <si>
-    <t>E11</t>
-  </si>
-  <si>
-    <t>E12</t>
-  </si>
-  <si>
-    <t>E13</t>
-  </si>
-  <si>
-    <t>E14</t>
-  </si>
-  <si>
-    <t>E15</t>
-  </si>
-  <si>
-    <t>E16</t>
-  </si>
-  <si>
-    <t>E18</t>
-  </si>
-  <si>
-    <t>E19</t>
-  </si>
-  <si>
-    <t>E20</t>
-  </si>
-  <si>
-    <t>E21</t>
-  </si>
-  <si>
-    <t>E22</t>
-  </si>
-  <si>
-    <t>E23</t>
-  </si>
-  <si>
-    <t>E24</t>
-  </si>
-  <si>
-    <t>E25</t>
-  </si>
-  <si>
-    <t>E27</t>
-  </si>
-  <si>
-    <t>E28</t>
-  </si>
-  <si>
-    <t>E29</t>
-  </si>
-  <si>
-    <t>E30</t>
-  </si>
-  <si>
-    <t>E31</t>
-  </si>
-  <si>
-    <t>E32</t>
-  </si>
-  <si>
-    <t>E33</t>
-  </si>
-  <si>
-    <t>E36</t>
-  </si>
-  <si>
-    <t>E37</t>
-  </si>
-  <si>
-    <t>E38</t>
-  </si>
-  <si>
-    <t>E39</t>
-  </si>
-  <si>
-    <t>E40</t>
-  </si>
-  <si>
-    <t>E41</t>
-  </si>
-  <si>
-    <t>E42</t>
-  </si>
-  <si>
-    <t>E43</t>
-  </si>
-  <si>
-    <t>E45</t>
-  </si>
-  <si>
-    <t>E46</t>
   </si>
 </sst>
 </file>
@@ -999,11 +777,13 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C4" t="s">
-        <v>58</v>
-      </c>
-      <c r="D4" t="s">
-        <v>95</v>
+      <c r="C4">
+        <f>F4</f>
+        <v>50</v>
+      </c>
+      <c r="D4" t="str">
+        <f t="shared" ref="D4:D9" si="0">G4</f>
+        <v>NA</v>
       </c>
       <c r="E4" t="s">
         <v>0</v>
@@ -1022,11 +802,13 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C5" t="s">
-        <v>59</v>
-      </c>
-      <c r="D5" t="s">
-        <v>96</v>
+      <c r="C5">
+        <f t="shared" ref="C5:C9" si="1">F5</f>
+        <v>62</v>
+      </c>
+      <c r="D5" t="str">
+        <f t="shared" si="0"/>
+        <v>NA</v>
       </c>
       <c r="E5" t="s">
         <v>1</v>
@@ -1045,11 +827,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C6" t="s">
-        <v>60</v>
-      </c>
-      <c r="D6" t="s">
-        <v>97</v>
+      <c r="C6">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="D6" t="str">
+        <f t="shared" si="0"/>
+        <v>NA</v>
       </c>
       <c r="E6" t="s">
         <v>2</v>
@@ -1068,11 +852,13 @@
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C7" t="s">
-        <v>61</v>
-      </c>
-      <c r="D7" t="s">
-        <v>98</v>
+      <c r="C7">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="D7" t="str">
+        <f t="shared" si="0"/>
+        <v>NA</v>
       </c>
       <c r="E7" t="s">
         <v>3</v>
@@ -1091,11 +877,13 @@
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C8" t="s">
-        <v>62</v>
-      </c>
-      <c r="D8" t="s">
-        <v>99</v>
+      <c r="C8">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="D8" t="str">
+        <f t="shared" si="0"/>
+        <v>NA</v>
       </c>
       <c r="E8" t="s">
         <v>4</v>
@@ -1114,11 +902,13 @@
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C9" t="s">
-        <v>63</v>
-      </c>
-      <c r="D9" t="s">
-        <v>100</v>
+      <c r="C9">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="D9" t="str">
+        <f t="shared" si="0"/>
+        <v>NA</v>
       </c>
       <c r="E9" t="s">
         <v>5</v>
@@ -1140,11 +930,13 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C11" t="s">
-        <v>64</v>
-      </c>
-      <c r="D11" t="s">
-        <v>101</v>
+      <c r="C11">
+        <f t="shared" ref="C11:C16" si="2">F11</f>
+        <v>50</v>
+      </c>
+      <c r="D11">
+        <f t="shared" ref="D11:D16" si="3">G11</f>
+        <v>50</v>
       </c>
       <c r="E11" t="s">
         <v>0</v>
@@ -1163,11 +955,13 @@
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C12" t="s">
-        <v>65</v>
-      </c>
-      <c r="D12" t="s">
-        <v>102</v>
+      <c r="C12">
+        <f t="shared" si="2"/>
+        <v>60</v>
+      </c>
+      <c r="D12">
+        <f t="shared" si="3"/>
+        <v>60</v>
       </c>
       <c r="E12" t="s">
         <v>1</v>
@@ -1186,11 +980,13 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C13" t="s">
-        <v>66</v>
-      </c>
-      <c r="D13" t="s">
-        <v>103</v>
+      <c r="C13">
+        <f t="shared" si="2"/>
+        <v>0.43</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="3"/>
+        <v>0.43</v>
       </c>
       <c r="E13" t="s">
         <v>17</v>
@@ -1209,11 +1005,13 @@
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C14" t="s">
-        <v>67</v>
-      </c>
-      <c r="D14" t="s">
-        <v>104</v>
+      <c r="C14">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="3"/>
+        <v>1</v>
       </c>
       <c r="E14" t="s">
         <v>18</v>
@@ -1232,11 +1030,13 @@
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C15" t="s">
-        <v>68</v>
-      </c>
-      <c r="D15" t="s">
-        <v>105</v>
+      <c r="C15">
+        <f t="shared" si="2"/>
+        <v>-3</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="3"/>
+        <v>-3</v>
       </c>
       <c r="E15" t="s">
         <v>19</v>
@@ -1255,11 +1055,13 @@
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C16" t="s">
-        <v>69</v>
-      </c>
-      <c r="D16" t="s">
-        <v>106</v>
+      <c r="C16">
+        <f t="shared" si="2"/>
+        <v>-3</v>
+      </c>
+      <c r="D16">
+        <f t="shared" si="3"/>
+        <v>-3</v>
       </c>
       <c r="E16" t="s">
         <v>20</v>
@@ -1283,11 +1085,13 @@
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C18" t="s">
-        <v>70</v>
-      </c>
-      <c r="D18" t="s">
-        <v>107</v>
+      <c r="C18">
+        <f t="shared" ref="C18:C25" si="4">F18</f>
+        <v>-3</v>
+      </c>
+      <c r="D18" t="str">
+        <f t="shared" ref="D18:D25" si="5">G18</f>
+        <v>NA</v>
       </c>
       <c r="E18" t="s">
         <v>22</v>
@@ -1307,11 +1111,13 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C19" t="s">
-        <v>71</v>
-      </c>
-      <c r="D19" t="s">
-        <v>108</v>
+      <c r="C19">
+        <f t="shared" si="4"/>
+        <v>9</v>
+      </c>
+      <c r="D19">
+        <f t="shared" si="5"/>
+        <v>9</v>
       </c>
       <c r="E19" t="s">
         <v>23</v>
@@ -1332,11 +1138,13 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C20" t="s">
-        <v>72</v>
-      </c>
-      <c r="D20" t="s">
-        <v>109</v>
+      <c r="C20">
+        <f t="shared" si="4"/>
+        <v>10</v>
+      </c>
+      <c r="D20">
+        <f t="shared" si="5"/>
+        <v>10</v>
       </c>
       <c r="E20" t="s">
         <v>24</v>
@@ -1357,11 +1165,13 @@
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C21" t="s">
-        <v>73</v>
-      </c>
-      <c r="D21" t="s">
-        <v>110</v>
+      <c r="C21">
+        <f t="shared" si="4"/>
+        <v>0.57000000000000006</v>
+      </c>
+      <c r="D21">
+        <f t="shared" si="5"/>
+        <v>0.57000000000000006</v>
       </c>
       <c r="E21" t="s">
         <v>25</v>
@@ -1382,11 +1192,13 @@
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C22" t="s">
-        <v>74</v>
-      </c>
-      <c r="D22" t="s">
-        <v>111</v>
+      <c r="C22">
+        <f t="shared" si="4"/>
+        <v>3.8778148173345128E-3</v>
+      </c>
+      <c r="D22">
+        <f t="shared" si="5"/>
+        <v>3.8778148173345128E-3</v>
       </c>
       <c r="E22" t="s">
         <v>26</v>
@@ -1407,11 +1219,13 @@
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C23" t="s">
-        <v>75</v>
-      </c>
-      <c r="D23" t="s">
-        <v>112</v>
+      <c r="C23">
+        <f t="shared" si="4"/>
+        <v>0.38778148173345128</v>
+      </c>
+      <c r="D23">
+        <f t="shared" si="5"/>
+        <v>0.38778148173345128</v>
       </c>
       <c r="E23" t="s">
         <v>27</v>
@@ -1432,11 +1246,13 @@
       </c>
     </row>
     <row r="24" spans="1:9" ht="18" x14ac:dyDescent="0.25">
-      <c r="C24" t="s">
-        <v>76</v>
-      </c>
-      <c r="D24" t="s">
-        <v>113</v>
+      <c r="C24">
+        <f t="shared" si="4"/>
+        <v>23.20894736842105</v>
+      </c>
+      <c r="D24">
+        <f t="shared" si="5"/>
+        <v>23.20894736842105</v>
       </c>
       <c r="E24" t="s">
         <v>28</v>
@@ -1457,11 +1273,13 @@
       </c>
     </row>
     <row r="25" spans="1:9" ht="18" x14ac:dyDescent="0.25">
-      <c r="C25" t="s">
-        <v>77</v>
-      </c>
-      <c r="D25" t="s">
-        <v>114</v>
+      <c r="C25">
+        <f t="shared" si="4"/>
+        <v>23.20894736842105</v>
+      </c>
+      <c r="D25" t="str">
+        <f t="shared" si="5"/>
+        <v>NA</v>
       </c>
       <c r="E25" t="s">
         <v>29</v>
@@ -1486,11 +1304,13 @@
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C27" t="s">
-        <v>78</v>
-      </c>
-      <c r="D27" t="s">
-        <v>115</v>
+      <c r="C27">
+        <f t="shared" ref="C27:C33" si="6">F27</f>
+        <v>0</v>
+      </c>
+      <c r="D27">
+        <f t="shared" ref="D27:D33" si="7">G27</f>
+        <v>0</v>
       </c>
       <c r="E27" t="s">
         <v>30</v>
@@ -1500,11 +1320,13 @@
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C28" t="s">
-        <v>79</v>
-      </c>
-      <c r="D28" t="s">
-        <v>116</v>
+      <c r="C28">
+        <f t="shared" si="6"/>
+        <v>50</v>
+      </c>
+      <c r="D28">
+        <f t="shared" si="7"/>
+        <v>50</v>
       </c>
       <c r="E28" t="s">
         <v>0</v>
@@ -1523,11 +1345,13 @@
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C29" t="s">
-        <v>80</v>
-      </c>
-      <c r="D29" t="s">
-        <v>117</v>
+      <c r="C29">
+        <f t="shared" si="6"/>
+        <v>60</v>
+      </c>
+      <c r="D29">
+        <f t="shared" si="7"/>
+        <v>60</v>
       </c>
       <c r="E29" t="s">
         <v>1</v>
@@ -1546,11 +1370,13 @@
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C30" t="s">
-        <v>81</v>
-      </c>
-      <c r="D30" t="s">
-        <v>118</v>
+      <c r="C30">
+        <f t="shared" si="6"/>
+        <v>0.43</v>
+      </c>
+      <c r="D30">
+        <f t="shared" si="7"/>
+        <v>0.43</v>
       </c>
       <c r="E30" t="s">
         <v>17</v>
@@ -1569,11 +1395,13 @@
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C31" t="s">
-        <v>82</v>
-      </c>
-      <c r="D31" t="s">
-        <v>119</v>
+      <c r="C31">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="D31">
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="E31" t="s">
         <v>31</v>
@@ -1592,11 +1420,13 @@
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C32" t="s">
-        <v>83</v>
-      </c>
-      <c r="D32" t="s">
-        <v>120</v>
+      <c r="C32">
+        <f t="shared" si="6"/>
+        <v>-3</v>
+      </c>
+      <c r="D32">
+        <f t="shared" si="7"/>
+        <v>-3</v>
       </c>
       <c r="E32" t="s">
         <v>19</v>
@@ -1615,11 +1445,13 @@
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C33" t="s">
-        <v>84</v>
-      </c>
-      <c r="D33" t="s">
-        <v>121</v>
+      <c r="C33">
+        <f t="shared" si="6"/>
+        <v>-3</v>
+      </c>
+      <c r="D33">
+        <f t="shared" si="7"/>
+        <v>-3</v>
       </c>
       <c r="E33" t="s">
         <v>20</v>
@@ -1643,11 +1475,13 @@
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C35" t="s">
-        <v>85</v>
-      </c>
-      <c r="D35" t="s">
-        <v>122</v>
+      <c r="C35">
+        <f t="shared" ref="C35:C42" si="8">F35</f>
+        <v>-3</v>
+      </c>
+      <c r="D35">
+        <f t="shared" ref="D35:D42" si="9">G35</f>
+        <v>-3</v>
       </c>
       <c r="E35" t="s">
         <v>32</v>
@@ -1668,11 +1502,13 @@
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C36" t="s">
-        <v>86</v>
-      </c>
-      <c r="D36" t="s">
-        <v>123</v>
+      <c r="C36">
+        <f t="shared" si="8"/>
+        <v>9</v>
+      </c>
+      <c r="D36">
+        <f t="shared" si="9"/>
+        <v>9</v>
       </c>
       <c r="E36" t="s">
         <v>23</v>
@@ -1693,11 +1529,13 @@
       </c>
     </row>
     <row r="37" spans="1:9" ht="18" x14ac:dyDescent="0.25">
-      <c r="C37" t="s">
-        <v>87</v>
-      </c>
-      <c r="D37" t="s">
-        <v>124</v>
+      <c r="C37">
+        <f t="shared" si="8"/>
+        <v>0.38778148173345128</v>
+      </c>
+      <c r="D37">
+        <f t="shared" si="9"/>
+        <v>0.38778148173345128</v>
       </c>
       <c r="E37" t="s">
         <v>36</v>
@@ -1718,11 +1556,13 @@
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C38" t="s">
-        <v>88</v>
-      </c>
-      <c r="D38" t="s">
-        <v>125</v>
+      <c r="C38">
+        <f t="shared" si="8"/>
+        <v>10</v>
+      </c>
+      <c r="D38">
+        <f t="shared" si="9"/>
+        <v>10</v>
       </c>
       <c r="E38" t="s">
         <v>24</v>
@@ -1743,11 +1583,13 @@
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C39" t="s">
-        <v>89</v>
-      </c>
-      <c r="D39" t="s">
-        <v>126</v>
+      <c r="C39">
+        <f t="shared" si="8"/>
+        <v>0.57000000000000006</v>
+      </c>
+      <c r="D39">
+        <f t="shared" si="9"/>
+        <v>0.57000000000000006</v>
       </c>
       <c r="E39" t="s">
         <v>33</v>
@@ -1768,11 +1610,13 @@
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C40" t="s">
-        <v>90</v>
-      </c>
-      <c r="D40" t="s">
-        <v>127</v>
+      <c r="C40">
+        <f t="shared" si="8"/>
+        <v>3.8778148173345128E-3</v>
+      </c>
+      <c r="D40">
+        <f t="shared" si="9"/>
+        <v>3.8778148173345128E-3</v>
       </c>
       <c r="E40" t="s">
         <v>47</v>
@@ -1793,11 +1637,13 @@
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C41" t="s">
-        <v>91</v>
-      </c>
-      <c r="D41" t="s">
-        <v>128</v>
+      <c r="C41">
+        <f t="shared" si="8"/>
+        <v>146.99</v>
+      </c>
+      <c r="D41">
+        <f t="shared" si="9"/>
+        <v>146.99</v>
       </c>
       <c r="E41" t="s">
         <v>34</v>
@@ -1818,11 +1664,13 @@
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C42" t="s">
-        <v>92</v>
-      </c>
-      <c r="D42" t="s">
-        <v>129</v>
+      <c r="C42">
+        <f t="shared" si="8"/>
+        <v>146.99</v>
+      </c>
+      <c r="D42" t="str">
+        <f t="shared" si="9"/>
+        <v>NA</v>
       </c>
       <c r="E42" t="s">
         <v>35</v>
@@ -1847,11 +1695,13 @@
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C44" t="s">
-        <v>93</v>
-      </c>
-      <c r="D44" t="s">
-        <v>130</v>
+      <c r="C44" t="str">
+        <f t="shared" ref="C44:C45" si="10">F44</f>
+        <v>Unknown Name</v>
+      </c>
+      <c r="D44" t="str">
+        <f t="shared" ref="D44:D45" si="11">G44</f>
+        <v>NA</v>
       </c>
       <c r="E44" t="s">
         <v>49</v>
@@ -1867,11 +1717,13 @@
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C45" t="s">
-        <v>94</v>
-      </c>
-      <c r="D45" t="s">
-        <v>131</v>
+      <c r="C45" t="str">
+        <f t="shared" si="10"/>
+        <v>%</v>
+      </c>
+      <c r="D45" t="str">
+        <f t="shared" si="11"/>
+        <v>NA</v>
       </c>
       <c r="E45" t="s">
         <v>51</v>

</xml_diff>